<commit_message>
docs: v2.8.17 登记——七面同步 + HANDOFF §12-75 九条判据 + ARCH_MAP §H9 #42 销账/§H10 锚复现 + 词汇表 159 条
两锚在定稿树各两轮 cmp 全等（B12 {"1":106,"2":194}／B11 {"1":108,"2":192}），
与 v2.8.16 的归一化输出只差两行且逐行点名＝npm 版本回显＋esbuild 体积行 ⇒ 容器层刀不动锚成立。
投影守卫本轮实证的目标换成"改了 md 忘记重跑"：把入库 xlsx 退回旧字节 ⇒ expected 27611 to be 28034 转红，重生成后 4/4 绿。
CI 状态暂标 PENDING，推送核验后回填。
</commit_message>
<xml_diff>
--- a/词汇表.xlsx
+++ b/词汇表.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="535" uniqueCount="363">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="541" uniqueCount="367">
   <si>
     <t>玩家词汇 · 大白话对照表（v2.8.14 界面口径）</t>
   </si>
@@ -48,7 +48,7 @@
     <t>一 棋盘与数字：30 条</t>
   </si>
   <si>
-    <t>二 行动按钮与提示：37 条</t>
+    <t>二 行动按钮与提示：38 条</t>
   </si>
   <si>
     <t>三 抽卡与开局：21 条</t>
@@ -60,7 +60,7 @@
     <t>五 结算录像日志：9 条</t>
   </si>
   <si>
-    <t>六 图鉴设置开发者：17 条</t>
+    <t>六 图鉴设置开发者：18 条</t>
   </si>
   <si>
     <t>七 界面里没有的词：8 条</t>
@@ -393,19 +393,19 @@
     <t>⏭️结束回合</t>
   </si>
   <si>
-    <t>我这回合到此为止。</t>
+    <t>我这回合到此为止。问话窗正开着时再点它＝等于「都不发动」，不会绕过窗。</t>
   </si>
   <si>
     <t>🌙 回合结束询问 · 是否发动将领技能？</t>
   </si>
   <si>
-    <t>回合收尾时问你一句：这些"回合结束时"技能要不要现在用。</t>
-  </si>
-  <si>
-    <t>⏭️ 跳过并结束回合</t>
-  </si>
-  <si>
-    <t>一个都不发动，直接收。</t>
+    <t>回合收尾时问你一句：这些"回合结束时"技能要不要现在用。问不问、列不列不能发动的，由对局设置里的「技能提示」两档决定（见 §六）。</t>
+  </si>
+  <si>
+    <t>🚫 都不发动</t>
+  </si>
+  <si>
+    <t>一个也不发动，直接结束本回合——这扇问话窗里唯一的出口（原先那个「⏭️ 跳过并结束回合（旧说法，已作废）」按钮已按 2.8.17 的裁决合并进来，只剩这一句）。</t>
   </si>
   <si>
     <t>⏳ 反应窗口开启 · 等待通过</t>
@@ -444,6 +444,12 @@
     <t>这个分支此刻不能选，原因写在冒号后面。</t>
   </si>
   <si>
+    <t>✕ {将名}【{技能名}】（本回合已发动过 / 不满足发动门槛：…）</t>
+  </si>
+  <si>
+    <t>「完整」档才出现的灰条：它只是告诉你为什么现在不能用，点它没有任何反应，也不算技能被拒绝——能不能发动从来由战场决定，不由这扇窗决定。</t>
+  </si>
+  <si>
     <t>⚡ {将名}【{技能名}】</t>
   </si>
   <si>
@@ -916,6 +922,12 @@
   </si>
   <si>
     <t>开着＝每次回合结束自动存一遍当前对局。</t>
+  </si>
+  <si>
+    <t>技能提示＝智能 / 完整（对局设置，2.8.17 起）</t>
+  </si>
+  <si>
+    <t>回合收尾时要不要停下来问你的档位。智能（默认）＝确实有能发动的才问，不能发动的不列；完整＝只要场上有"回合结束时"技能就问，暂时不能发动的也列出来并写明原因。两档都不改变技能本身能不能发动，也不影响录像。</t>
   </si>
   <si>
     <t>你以为有的词</t>
@@ -1981,7 +1993,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -2404,6 +2416,17 @@
         <v>152</v>
       </c>
       <c r="C38" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="C39" s="3" t="s">
         <v>1</v>
       </c>
     </row>
@@ -2436,10 +2459,10 @@
     </row>
     <row r="2" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>1</v>
@@ -2447,10 +2470,10 @@
     </row>
     <row r="3" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>1</v>
@@ -2458,21 +2481,21 @@
     </row>
     <row r="4" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="5" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>1</v>
@@ -2480,10 +2503,10 @@
     </row>
     <row r="6" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>1</v>
@@ -2491,10 +2514,10 @@
     </row>
     <row r="7" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>1</v>
@@ -2502,10 +2525,10 @@
     </row>
     <row r="8" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>1</v>
@@ -2513,10 +2536,10 @@
     </row>
     <row r="9" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>1</v>
@@ -2524,10 +2547,10 @@
     </row>
     <row r="10" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>1</v>
@@ -2535,10 +2558,10 @@
     </row>
     <row r="11" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>1</v>
@@ -2546,10 +2569,10 @@
     </row>
     <row r="12" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>1</v>
@@ -2557,10 +2580,10 @@
     </row>
     <row r="13" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>1</v>
@@ -2568,10 +2591,10 @@
     </row>
     <row r="14" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>1</v>
@@ -2579,10 +2602,10 @@
     </row>
     <row r="15" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>1</v>
@@ -2590,10 +2613,10 @@
     </row>
     <row r="16" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C16" s="3" t="s">
         <v>1</v>
@@ -2601,10 +2624,10 @@
     </row>
     <row r="17" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>1</v>
@@ -2612,10 +2635,10 @@
     </row>
     <row r="18" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>1</v>
@@ -2623,10 +2646,10 @@
     </row>
     <row r="19" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>1</v>
@@ -2634,10 +2657,10 @@
     </row>
     <row r="20" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>1</v>
@@ -2645,10 +2668,10 @@
     </row>
     <row r="21" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>1</v>
@@ -2656,10 +2679,10 @@
     </row>
     <row r="22" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C22" s="3" t="s">
         <v>1</v>
@@ -2694,10 +2717,10 @@
     </row>
     <row r="2" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>1</v>
@@ -2705,10 +2728,10 @@
     </row>
     <row r="3" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>1</v>
@@ -2716,10 +2739,10 @@
     </row>
     <row r="4" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>1</v>
@@ -2727,10 +2750,10 @@
     </row>
     <row r="5" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>1</v>
@@ -2738,10 +2761,10 @@
     </row>
     <row r="6" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>1</v>
@@ -2749,10 +2772,10 @@
     </row>
     <row r="7" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>1</v>
@@ -2760,10 +2783,10 @@
     </row>
     <row r="8" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>1</v>
@@ -2771,10 +2794,10 @@
     </row>
     <row r="9" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>1</v>
@@ -2782,10 +2805,10 @@
     </row>
     <row r="10" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>1</v>
@@ -2793,10 +2816,10 @@
     </row>
     <row r="11" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>1</v>
@@ -2804,10 +2827,10 @@
     </row>
     <row r="12" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>1</v>
@@ -2815,10 +2838,10 @@
     </row>
     <row r="13" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>1</v>
@@ -2826,10 +2849,10 @@
     </row>
     <row r="14" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>1</v>
@@ -2837,10 +2860,10 @@
     </row>
     <row r="15" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>1</v>
@@ -2848,10 +2871,10 @@
     </row>
     <row r="16" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C16" s="3" t="s">
         <v>1</v>
@@ -2859,10 +2882,10 @@
     </row>
     <row r="17" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>1</v>
@@ -2870,10 +2893,10 @@
     </row>
     <row r="18" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>1</v>
@@ -2881,10 +2904,10 @@
     </row>
     <row r="19" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>1</v>
@@ -2892,10 +2915,10 @@
     </row>
     <row r="20" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="C20" s="3" t="s">
         <v>1</v>
@@ -2903,10 +2926,10 @@
     </row>
     <row r="21" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>1</v>
@@ -2914,10 +2937,10 @@
     </row>
     <row r="22" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C22" s="3" t="s">
         <v>1</v>
@@ -2925,10 +2948,10 @@
     </row>
     <row r="23" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="C23" s="3" t="s">
         <v>1</v>
@@ -2936,10 +2959,10 @@
     </row>
     <row r="24" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>1</v>
@@ -2947,10 +2970,10 @@
     </row>
     <row r="25" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>1</v>
@@ -2958,10 +2981,10 @@
     </row>
     <row r="26" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>1</v>
@@ -2969,7 +2992,7 @@
     </row>
     <row r="28" spans="1:3" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B28" s="6"/>
       <c r="C28" s="6"/>
@@ -3006,10 +3029,10 @@
     </row>
     <row r="2" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>1</v>
@@ -3017,10 +3040,10 @@
     </row>
     <row r="3" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>1</v>
@@ -3028,10 +3051,10 @@
     </row>
     <row r="4" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>1</v>
@@ -3039,10 +3062,10 @@
     </row>
     <row r="5" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>1</v>
@@ -3050,10 +3073,10 @@
     </row>
     <row r="6" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>1</v>
@@ -3061,10 +3084,10 @@
     </row>
     <row r="7" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>1</v>
@@ -3072,10 +3095,10 @@
     </row>
     <row r="8" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>1</v>
@@ -3083,10 +3106,10 @@
     </row>
     <row r="9" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>1</v>
@@ -3094,10 +3117,10 @@
     </row>
     <row r="10" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>1</v>
@@ -3111,7 +3134,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -3132,10 +3155,10 @@
     </row>
     <row r="2" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>1</v>
@@ -3143,10 +3166,10 @@
     </row>
     <row r="3" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>1</v>
@@ -3154,10 +3177,10 @@
     </row>
     <row r="4" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>1</v>
@@ -3165,10 +3188,10 @@
     </row>
     <row r="5" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>1</v>
@@ -3176,10 +3199,10 @@
     </row>
     <row r="6" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>1</v>
@@ -3187,10 +3210,10 @@
     </row>
     <row r="7" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>1</v>
@@ -3198,10 +3221,10 @@
     </row>
     <row r="8" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>1</v>
@@ -3209,10 +3232,10 @@
     </row>
     <row r="9" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>1</v>
@@ -3220,10 +3243,10 @@
     </row>
     <row r="10" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>1</v>
@@ -3231,10 +3254,10 @@
     </row>
     <row r="11" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="C11" s="3" t="s">
         <v>1</v>
@@ -3242,10 +3265,10 @@
     </row>
     <row r="12" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>1</v>
@@ -3253,10 +3276,10 @@
     </row>
     <row r="13" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>1</v>
@@ -3264,10 +3287,10 @@
     </row>
     <row r="14" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="C14" s="3" t="s">
         <v>1</v>
@@ -3275,10 +3298,10 @@
     </row>
     <row r="15" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>1</v>
@@ -3286,10 +3309,10 @@
     </row>
     <row r="16" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="C16" s="3" t="s">
         <v>1</v>
@@ -3297,10 +3320,10 @@
     </row>
     <row r="17" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>1</v>
@@ -3308,12 +3331,23 @@
     </row>
     <row r="18" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="C18" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>301</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>302</v>
+      </c>
+      <c r="C19" s="3" t="s">
         <v>1</v>
       </c>
     </row>
@@ -3335,10 +3369,10 @@
   <sheetData>
     <row r="1" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="C1" s="5" t="s">
         <v>18</v>
@@ -3346,10 +3380,10 @@
     </row>
     <row r="2" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>302</v>
+        <v>306</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>1</v>
@@ -3357,10 +3391,10 @@
     </row>
     <row r="3" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>1</v>
@@ -3368,10 +3402,10 @@
     </row>
     <row r="4" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>306</v>
+        <v>310</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>1</v>
@@ -3379,10 +3413,10 @@
     </row>
     <row r="5" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>1</v>
@@ -3390,10 +3424,10 @@
     </row>
     <row r="6" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>1</v>
@@ -3401,10 +3435,10 @@
     </row>
     <row r="7" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>311</v>
+        <v>315</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>1</v>
@@ -3412,10 +3446,10 @@
     </row>
     <row r="8" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>313</v>
+        <v>317</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>314</v>
+        <v>318</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>1</v>
@@ -3423,10 +3457,10 @@
     </row>
     <row r="9" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>1</v>
@@ -3451,50 +3485,50 @@
   <sheetData>
     <row r="1" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>318</v>
+        <v>322</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>320</v>
+        <v>324</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>321</v>
+        <v>325</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>322</v>
+        <v>326</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>329</v>
+        <v>333</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>330</v>
+        <v>334</v>
       </c>
       <c r="E3" s="3" t="s">
         <v>1</v>
@@ -3502,16 +3536,16 @@
     </row>
     <row r="4" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>331</v>
+        <v>335</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>333</v>
+        <v>337</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>334</v>
+        <v>338</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>1</v>
@@ -3519,16 +3553,16 @@
     </row>
     <row r="5" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>336</v>
+        <v>340</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>337</v>
+        <v>341</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>1</v>
@@ -3536,16 +3570,16 @@
     </row>
     <row r="6" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>1</v>
@@ -3553,16 +3587,16 @@
     </row>
     <row r="7" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>343</v>
+        <v>347</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>1</v>
@@ -3570,16 +3604,16 @@
     </row>
     <row r="8" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>347</v>
+        <v>351</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>350</v>
+        <v>354</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>1</v>
@@ -3587,16 +3621,16 @@
     </row>
     <row r="9" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>351</v>
+        <v>355</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>352</v>
+        <v>356</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>1</v>
@@ -3604,16 +3638,16 @@
     </row>
     <row r="10" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>357</v>
+        <v>361</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>358</v>
+        <v>362</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>1</v>
@@ -3621,16 +3655,16 @@
     </row>
     <row r="11" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>359</v>
+        <v>363</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>362</v>
+        <v>366</v>
       </c>
       <c r="E11" s="3" t="s">
         <v>1</v>

</xml_diff>